<commit_message>
Add baseline HbA1c and BMI from observations to Table 1 and PS models
</commit_message>
<xml_diff>
--- a/reports/Table1_Baseline.xlsx
+++ b/reports/Table1_Baseline.xlsx
@@ -434,11 +434,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I21"/>
+  <dimension ref="A1:I27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="27" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="33" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
@@ -663,75 +663,75 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Demographics</t>
+          <t>Clinical measurements</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Gender: F</t>
+          <t>HbA1c (%) — mean (SD)</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>24 (49.0%)</t>
+          <t>7.4 (0.5)</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>13 (65.0%)</t>
+          <t>7.0 (0.2)</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>37 (53.6%)</t>
+          <t>7.3 (0.5)</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>-0.322</v>
+        <v>1.157</v>
       </c>
       <c r="G7" t="b">
         <v>0</v>
       </c>
       <c r="H7" t="n">
-        <v>0.3448</v>
+        <v>0.0024</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>NS</t>
+          <t>**</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Demographics</t>
+          <t>Clinical measurements</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Gender: M</t>
+          <t>HbA1c (%) — median (IQR)</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>25 (51.0%)</t>
+          <t>7.5 (7.5–7.6)</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>7 (35.0%)</t>
+          <t>6.9 (6.9–7.0)</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>32 (46.4%)</t>
+          <t>7.5 (6.9–7.6)</t>
         </is>
       </c>
       <c r="F8" t="n">
-        <v>0.322</v>
-      </c>
-      <c r="G8" t="b">
-        <v>0</v>
+        <v/>
+      </c>
+      <c r="G8" t="n">
+        <v/>
       </c>
       <c r="H8" t="n">
         <v/>
@@ -743,114 +743,114 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Demographics</t>
+          <t>Clinical measurements</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Race: asian</t>
+          <t>HbA1c (%) — missing, n</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>1 (2.0%)</t>
+          <t>31</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>0 (0.0%)</t>
+          <t>13</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1 (1.4%)</t>
+          <t>44</t>
         </is>
       </c>
       <c r="F9" t="n">
-        <v>0.202</v>
-      </c>
-      <c r="G9" t="b">
-        <v>0</v>
+        <v/>
+      </c>
+      <c r="G9" t="n">
+        <v/>
       </c>
       <c r="H9" t="n">
-        <v>0.4631</v>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>NS</t>
-        </is>
+        <v/>
+      </c>
+      <c r="I9" t="n">
+        <v/>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Demographics</t>
+          <t>Clinical measurements</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Race: black</t>
+          <t>BMI (kg/m2) — mean (SD)</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2 (4.1%)</t>
+          <t>30.3 (0.5)</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>3 (15.0%)</t>
+          <t>30.7 (5.3)</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>5 (7.2%)</t>
+          <t>30.4 (2.7)</t>
         </is>
       </c>
       <c r="F10" t="n">
-        <v>-0.37</v>
+        <v>-0.108</v>
       </c>
       <c r="G10" t="b">
         <v>0</v>
       </c>
       <c r="H10" t="n">
-        <v/>
-      </c>
-      <c r="I10" t="n">
-        <v/>
+        <v>0.1071</v>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>NS</t>
+        </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Demographics</t>
+          <t>Clinical measurements</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Race: hawaiian</t>
+          <t>BMI (kg/m2) — median (IQR)</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>1 (2.0%)</t>
+          <t>30.2 (30.1–30.4)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>0 (0.0%)</t>
+          <t>27.8 (27.6–32.6)</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>1 (1.4%)</t>
+          <t>30.2 (30.0–30.4)</t>
         </is>
       </c>
       <c r="F11" t="n">
-        <v>0.202</v>
-      </c>
-      <c r="G11" t="b">
-        <v>0</v>
+        <v/>
+      </c>
+      <c r="G11" t="n">
+        <v/>
       </c>
       <c r="H11" t="n">
         <v/>
@@ -862,34 +862,34 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Demographics</t>
+          <t>Clinical measurements</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Race: native</t>
+          <t>BMI (kg/m2) — missing, n</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>1 (2.0%)</t>
+          <t>31</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>0 (0.0%)</t>
+          <t>13</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>1 (1.4%)</t>
+          <t>44</t>
         </is>
       </c>
       <c r="F12" t="n">
-        <v>0.202</v>
-      </c>
-      <c r="G12" t="b">
-        <v>0</v>
+        <v/>
+      </c>
+      <c r="G12" t="n">
+        <v/>
       </c>
       <c r="H12" t="n">
         <v/>
@@ -906,112 +906,112 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Race: white</t>
+          <t xml:space="preserve">  Gender: F</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>44 (89.8%)</t>
+          <t>24 (49.0%)</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>17 (85.0%)</t>
+          <t>13 (65.0%)</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>61 (88.4%)</t>
+          <t>37 (53.6%)</t>
         </is>
       </c>
       <c r="F13" t="n">
-        <v>0.142</v>
+        <v>-0.322</v>
       </c>
       <c r="G13" t="b">
         <v>0</v>
       </c>
       <c r="H13" t="n">
-        <v/>
-      </c>
-      <c r="I13" t="n">
-        <v/>
+        <v>0.3448</v>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>NS</t>
+        </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Clinical characteristics</t>
+          <t>Demographics</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Hypertension</t>
+          <t xml:space="preserve">  Gender: M</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>27 (55.1%)</t>
+          <t>25 (51.0%)</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>12 (60.0%)</t>
+          <t>7 (35.0%)</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>39 (56.5%)</t>
+          <t>32 (46.4%)</t>
         </is>
       </c>
       <c r="F14" t="n">
-        <v>-0.097</v>
+        <v>0.322</v>
       </c>
       <c r="G14" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H14" t="n">
-        <v>0.9166</v>
-      </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>NS</t>
-        </is>
+        <v/>
+      </c>
+      <c r="I14" t="n">
+        <v/>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Clinical characteristics</t>
+          <t>Demographics</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Hyperlipidemia</t>
+          <t xml:space="preserve">  Race: asian</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>8 (16.3%)</t>
+          <t>1 (2.0%)</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>4 (20.0%)</t>
+          <t>0 (0.0%)</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>12 (17.4%)</t>
+          <t>1 (1.4%)</t>
         </is>
       </c>
       <c r="F15" t="n">
-        <v>-0.094</v>
+        <v>0.202</v>
       </c>
       <c r="G15" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H15" t="n">
-        <v>0.7343</v>
+        <v>0.4631</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
@@ -1022,165 +1022,157 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Clinical characteristics</t>
+          <t>Demographics</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Obesity</t>
+          <t xml:space="preserve">  Race: black</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>49 (100.0%)</t>
+          <t>2 (4.1%)</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>14 (70.0%)</t>
+          <t>3 (15.0%)</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>63 (91.3%)</t>
+          <t>5 (7.2%)</t>
         </is>
       </c>
       <c r="F16" t="n">
-        <v>0.902</v>
+        <v>-0.37</v>
       </c>
       <c r="G16" t="b">
         <v>0</v>
       </c>
       <c r="H16" t="n">
-        <v>0.0003</v>
-      </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>***</t>
-        </is>
+        <v/>
+      </c>
+      <c r="I16" t="n">
+        <v/>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Clinical characteristics</t>
+          <t>Demographics</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Cardiovascular disease</t>
+          <t xml:space="preserve">  Race: hawaiian</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>11 (22.4%)</t>
+          <t>1 (2.0%)</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>10 (50.0%)</t>
+          <t>0 (0.0%)</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>21 (30.4%)</t>
+          <t>1 (1.4%)</t>
         </is>
       </c>
       <c r="F17" t="n">
-        <v>-0.587</v>
+        <v>0.202</v>
       </c>
       <c r="G17" t="b">
         <v>0</v>
       </c>
       <c r="H17" t="n">
-        <v>0.049</v>
-      </c>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>*</t>
-        </is>
+        <v/>
+      </c>
+      <c r="I17" t="n">
+        <v/>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Clinical characteristics</t>
+          <t>Demographics</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Chronic kidney disease</t>
+          <t xml:space="preserve">  Race: native</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>7 (14.3%)</t>
+          <t>1 (2.0%)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>13 (65.0%)</t>
+          <t>0 (0.0%)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>20 (29.0%)</t>
+          <t>1 (1.4%)</t>
         </is>
       </c>
       <c r="F18" t="n">
-        <v>-1.188</v>
+        <v>0.202</v>
       </c>
       <c r="G18" t="b">
         <v>0</v>
       </c>
       <c r="H18" t="n">
-        <v>0.0001</v>
-      </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>***</t>
-        </is>
+        <v/>
+      </c>
+      <c r="I18" t="n">
+        <v/>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Clinical characteristics</t>
+          <t>Demographics</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Diabetic nephropathy</t>
+          <t xml:space="preserve">  Race: white</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>7 (14.3%)</t>
+          <t>44 (89.8%)</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>16 (80.0%)</t>
+          <t>17 (85.0%)</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>23 (33.3%)</t>
+          <t>61 (88.4%)</t>
         </is>
       </c>
       <c r="F19" t="n">
-        <v>-1.716</v>
+        <v>0.142</v>
       </c>
       <c r="G19" t="b">
         <v>0</v>
       </c>
       <c r="H19" t="n">
-        <v>0</v>
-      </c>
-      <c r="I19" t="inlineStr">
-        <is>
-          <t>***</t>
-        </is>
+        <v/>
+      </c>
+      <c r="I19" t="n">
+        <v/>
       </c>
     </row>
     <row r="20">
@@ -1191,32 +1183,32 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Diabetic neuropathy</t>
+          <t>Hypertension</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>5 (10.2%)</t>
+          <t>27 (55.1%)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>5 (25.0%)</t>
+          <t>12 (60.0%)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>10 (14.5%)</t>
+          <t>39 (56.5%)</t>
         </is>
       </c>
       <c r="F20" t="n">
-        <v>-0.388</v>
+        <v>-0.097</v>
       </c>
       <c r="G20" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H20" t="n">
-        <v>0.1399</v>
+        <v>0.9166</v>
       </c>
       <c r="I20" t="inlineStr">
         <is>
@@ -1232,34 +1224,280 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
+          <t>Hyperlipidemia</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>8 (16.3%)</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>4 (20.0%)</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>12 (17.4%)</t>
+        </is>
+      </c>
+      <c r="F21" t="n">
+        <v>-0.094</v>
+      </c>
+      <c r="G21" t="b">
+        <v>1</v>
+      </c>
+      <c r="H21" t="n">
+        <v>0.7343</v>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>NS</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Clinical characteristics</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Obesity</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>49 (100.0%)</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>14 (70.0%)</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>63 (91.3%)</t>
+        </is>
+      </c>
+      <c r="F22" t="n">
+        <v>0.902</v>
+      </c>
+      <c r="G22" t="b">
+        <v>0</v>
+      </c>
+      <c r="H22" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>***</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Clinical characteristics</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Cardiovascular disease</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>11 (22.4%)</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>10 (50.0%)</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>21 (30.4%)</t>
+        </is>
+      </c>
+      <c r="F23" t="n">
+        <v>-0.587</v>
+      </c>
+      <c r="G23" t="b">
+        <v>0</v>
+      </c>
+      <c r="H23" t="n">
+        <v>0.049</v>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Clinical characteristics</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Chronic kidney disease</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>7 (14.3%)</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>13 (65.0%)</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>20 (29.0%)</t>
+        </is>
+      </c>
+      <c r="F24" t="n">
+        <v>-1.188</v>
+      </c>
+      <c r="G24" t="b">
+        <v>0</v>
+      </c>
+      <c r="H24" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>***</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Clinical characteristics</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Diabetic nephropathy</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>7 (14.3%)</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>16 (80.0%)</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>23 (33.3%)</t>
+        </is>
+      </c>
+      <c r="F25" t="n">
+        <v>-1.716</v>
+      </c>
+      <c r="G25" t="b">
+        <v>0</v>
+      </c>
+      <c r="H25" t="n">
+        <v>0</v>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>***</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Clinical characteristics</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Diabetic neuropathy</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>5 (10.2%)</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>5 (25.0%)</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>10 (14.5%)</t>
+        </is>
+      </c>
+      <c r="F26" t="n">
+        <v>-0.388</v>
+      </c>
+      <c r="G26" t="b">
+        <v>0</v>
+      </c>
+      <c r="H26" t="n">
+        <v>0.1399</v>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>NS</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Clinical characteristics</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
           <t>Diabetic retinopathy</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="C27" t="inlineStr">
         <is>
           <t>1 (2.0%)</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
+      <c r="D27" t="inlineStr">
         <is>
           <t>1 (5.0%)</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr">
+      <c r="E27" t="inlineStr">
         <is>
           <t>2 (2.9%)</t>
         </is>
       </c>
-      <c r="F21" t="n">
+      <c r="F27" t="n">
         <v>-0.158</v>
       </c>
-      <c r="G21" t="b">
-        <v>0</v>
-      </c>
-      <c r="H21" t="n">
+      <c r="G27" t="b">
+        <v>0</v>
+      </c>
+      <c r="H27" t="n">
         <v>0.4987</v>
       </c>
-      <c r="I21" t="inlineStr">
+      <c r="I27" t="inlineStr">
         <is>
           <t>NS</t>
         </is>

</xml_diff>